<commit_message>
Leads: 2026-10-31 05:03 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -594,7 +594,6 @@
           <t>info@goliathroofingofflorida.com</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Miramar FL</t>
@@ -614,6 +613,66 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Grand Prairie, Texas Roofing Company | Birdcreek Roofing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>birdcreekroofing.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.birdcreekroofing.com/service-area/Grand-Prairie-Texas-Roofing-Company</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Roofing Hail</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>admin@birdcreekroofing.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>800-693-6041</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>residential roofing company Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-10-31</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-31 05:06 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BMC Installation Heating &amp; Air Conditioning Inc | Silver Spring, MD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>bmcmyers.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.bmcmyers.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Hours Mon</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>bmcjohns@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>301-562-9008</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Silver Spring MD</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>HVAC contractor Silver Spring MD</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-31 05:07 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,126 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Regal Construction</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>regalconstruction.us</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.regalconstruction.us/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Mark Tarnowsky</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@regalconstruction.us</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>501-366-5246</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Little Rock AR</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roofing contractor Little Rock AR</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Roof Repair Fontana, CA | Fast &amp; Reliable | All Seasons Roofing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>allseasonsroofexperts.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://allseasonsroofexperts.com/roof-repair-fontana-ca</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>contact@allseasonsroofexperts.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(909) 503-4841</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Fontana CA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roof repair company Fontana CA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-31 05:09 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -858,6 +858,62 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HVAC Experts Ann Arbor - Comfort Mechanical Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>comfortmechanicalhvac.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://comfortmechanicalhvac.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>comfortmechanicalheatingandac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>7343408364</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>74</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>heating and cooling company Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-31 05:12 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -879,7 +879,6 @@
           <t>https://comfortmechanicalhvac.com/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>comfortmechanicalheatingandac@gmail.com</t>
@@ -909,6 +908,62 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Roofing in Sterling Heights, MI | Constantine Roofing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>constantineroofing.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.constantineroofing.com/roofing-in-sterling-heights</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>michelle@constantineroofing.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(586) 726-9931</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>86</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roof repair company Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-10-31</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-31 14:26 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -934,7 +934,6 @@
           <t>https://www.constantineroofing.com/roofing-in-sterling-heights</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>michelle@constantineroofing.com</t>
@@ -964,6 +963,242 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>The Plumber Leads</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>theplumberone.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.theplumberone.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Owner Operated</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@mysite.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>831-737-9032</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>plumber Salinas CA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Baseline Coatings</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>baselinecoatings.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://baselinecoatings.com/locations/columbus-ga/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Google Rating</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@baselinecoatings.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(706) 562-4656</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Columbus GA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roofing contractor Columbus GA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Idaho Falls Plumbing Company</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>idahofallsplumbingcompany.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://idahofallsplumbingcompany.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>yourifplumber@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>208-569-9743</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>plumbing company Idaho Falls ID</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hutch's Plumbing - Plumber and Heating Technician | Salinas, CA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>plumbersalinas.net</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.plumbersalinas.net/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Monterey County</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>hutchplumb@sbcglobal.net</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>831-754-3740</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>86</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>plumber Salinas CA</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-31</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-31 14:27 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1109,7 +1109,6 @@
           <t>https://idahofallsplumbingcompany.com/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>yourifplumber@gmail.com</t>
@@ -1199,6 +1198,62 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Electrician &amp; HVAC Contractor in Queens, NY</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>aproelectricalhvac.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://aproelectricalhvac.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>aproelectricalinc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(929) 529-3465</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>80</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>HVAC contractor Queens NY</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-10-31</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-31 14:33 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1224,7 +1224,6 @@
           <t>https://aproelectricalhvac.com/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>aproelectricalinc@gmail.com</t>
@@ -1254,6 +1253,66 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ready Energy Solutions</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>readyenergyhvac.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.readyenergyhvac.com/federal-way/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Alex Stelmakh</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>readyenergyllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(206) 750-7020</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Federal Way WA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>furnace repair Federal Way WA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>2026-10-31</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-31 14:36 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1318,6 +1318,122 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HVAC Services Sunnyvale | Balcom Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>balcomair.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://balcomair.com/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>balcomair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>408-307-3413</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Sunnyvale CA</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>HVAC contractor Sunnyvale CA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Therma Tech Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>thermatechhvac.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://thermatechhvac.com/service-area/sunnyvale</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sunnyvale Therma</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@thermatechhvac.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>408-629-5400</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Sunnyvale CA</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>HVAC contractor Sunnyvale CA</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-31 14:41 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1339,7 +1339,6 @@
           <t>https://balcomair.com/</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>balcomair@gmail.com</t>
@@ -1429,6 +1428,122 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Renton, WA | ACN Roof LLC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>acnproroofing.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://acnproroofing.com/roof-replacement-renton-wa</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Pacific Northwest</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>acnnewroof@gmail.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(425) 207-6771</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Renton WA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>roof replacement Renton WA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Water Heater Repair in Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.apgplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.apgplumbingservices.com/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>contact@apgplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(888) 576-6192</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>90</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>water heater repair Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-10-31</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-31 14:47 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-31.xlsx
+++ b/output/leads_2026-10-31.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1514,7 +1514,6 @@
           <t>https://aberdeen-sd.apgplumbingservices.com/water-heater-repair/</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>contact@apgplumbingservices.com</t>
@@ -1544,6 +1543,66 @@
         </is>
       </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Proud American Roofing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>proudamericanroof.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://proudamericanroof.com/pages/lakeland</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Like Family</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>wecare@chooseproud.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(813)-500-2004</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>roof replacement Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>2026-10-31</t>
         </is>

</xml_diff>